<commit_message>
feat(roster): SEC Burger/Overton, alias coverage, data-dir source of truth
- Add Nandre Burger and Craig Overton to SEC squad (full-name-only
  alias patterns to avoid false positives)
- Expand PLAYER_ALIASES coverage across all four franchises
- Canonical roster at data/squadofsunrisers.xlsx with root fallback;
  sync script writes both copies (90 rows, Leeds Women preserved)
</commit_message>
<xml_diff>
--- a/squadofsunrisers.xlsx
+++ b/squadofsunrisers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2663,6 +2663,56 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Sunrisers Eastern Cape SA20 2026</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Nandre Burger</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Bowler</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Sunrisers Eastern Cape SA20 2026</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Craig Overton</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>All-rounder</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Overseas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>